<commit_message>
Lock template cells and keep dropdowns
Protect the Course Records worksheet so headers, banner, and the
Instructions tab are read-only while only the data-entry cells remain
editable. Row insertion/deletion stays enabled and the Course Type,
Time Zone, and State dropdowns continue to work under protection.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y8EAvR5NE5imEw4oAyMGQu
</commit_message>
<xml_diff>
--- a/Course-Records-Upload-Template.xlsx
+++ b/Course-Records-Upload-Template.xlsx
@@ -134,11 +134,13 @@
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="4" fillId="4" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" applyAlignment="1" applyProtection="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment vertical="center" wrapText="1"/>
+      <protection locked="0" hidden="0"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="left" vertical="center" wrapText="1" indent="1"/>
@@ -673,7 +675,7 @@
     <row r="2" ht="30" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>Fill in one course per row starting at row 5. Columns marked with * are required. Row 4 is a filled-in example — you may delete it before uploading. See the Instructions tab for details.</t>
+          <t>Fill in one course per row starting at row 5. Columns marked with * are required. Only the data cells (rows 4 and below) are editable — headers and instructions are locked. Row 4 is an example you can overwrite. See the Instructions tab for details.</t>
         </is>
       </c>
     </row>
@@ -5093,6 +5095,7 @@
       <c r="S205" s="6" t="n"/>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="0"/>
   <mergeCells count="2">
     <mergeCell ref="A2:S2"/>
     <mergeCell ref="A1:S1"/>
@@ -5570,6 +5573,7 @@
       </c>
     </row>
   </sheetData>
+  <sheetProtection selectLockedCells="1" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <mergeCells count="11">
     <mergeCell ref="B30:C30"/>
     <mergeCell ref="B33:C33"/>

</xml_diff>

<commit_message>
Add Provider column to course upload template
Add a Provider column (free text) so uploads can specify the offering
provider by name. It must match an existing provider; left blank, the
upload uses the uploader's own provider. Update the example row and
Instructions tab accordingly.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y8EAvR5NE5imEw4oAyMGQu
</commit_message>
<xml_diff>
--- a/Course-Records-Upload-Template.xlsx
+++ b/Course-Records-Upload-Template.xlsx
@@ -265,80 +265,85 @@
     </comment>
     <comment ref="D3" authorId="0" shapeId="0">
       <text>
-        <t>Choose one from the dropdown. Required.</t>
+        <t>The provider/organization offering the course. Must exactly match an existing provider name. Leave blank to use the uploader's own provider.</t>
       </text>
     </comment>
     <comment ref="E3" authorId="0" shapeId="0">
       <text>
-        <t>Format MM/DD/YYYY. Required.</t>
+        <t>Choose one from the dropdown. Required.</t>
       </text>
     </comment>
     <comment ref="F3" authorId="0" shapeId="0">
       <text>
-        <t>Format H:MM AM/PM, e.g. 9:00 AM. Required.</t>
+        <t>Format MM/DD/YYYY. Required.</t>
       </text>
     </comment>
     <comment ref="G3" authorId="0" shapeId="0">
       <text>
-        <t>Choose one from the dropdown. Applies to all times in the row. Required.</t>
+        <t>Format H:MM AM/PM, e.g. 9:00 AM. Required.</t>
       </text>
     </comment>
     <comment ref="H3" authorId="0" shapeId="0">
       <text>
-        <t>Optional. For multi-day courses. MM/DD/YYYY.</t>
+        <t>Choose one from the dropdown. Applies to all times in the row. Required.</t>
       </text>
     </comment>
     <comment ref="I3" authorId="0" shapeId="0">
       <text>
-        <t>Optional. H:MM AM/PM.</t>
+        <t>Optional. For multi-day courses. MM/DD/YYYY.</t>
       </text>
     </comment>
     <comment ref="J3" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Must be before Start Date. MM/DD/YYYY.</t>
+        <t>Optional. H:MM AM/PM.</t>
       </text>
     </comment>
     <comment ref="K3" authorId="0" shapeId="0">
       <text>
-        <t>Optional. H:MM AM/PM.</t>
+        <t>Optional. Must be before Start Date. MM/DD/YYYY.</t>
       </text>
     </comment>
     <comment ref="L3" authorId="0" shapeId="0">
       <text>
-        <t>Venue or meeting place name. Required.</t>
+        <t>Optional. H:MM AM/PM.</t>
       </text>
     </comment>
     <comment ref="M3" authorId="0" shapeId="0">
       <text>
-        <t>Optional street address.</t>
+        <t>Venue or meeting place name. Required.</t>
       </text>
     </comment>
     <comment ref="N3" authorId="0" shapeId="0">
       <text>
-        <t>Optional.</t>
+        <t>Optional street address.</t>
       </text>
     </comment>
     <comment ref="O3" authorId="0" shapeId="0">
       <text>
-        <t>Two-letter code from dropdown. Required.</t>
+        <t>Optional.</t>
       </text>
     </comment>
     <comment ref="P3" authorId="0" shapeId="0">
       <text>
-        <t>Optional. 5 digits (or 5+4).</t>
+        <t>Two-letter code from dropdown. Required.</t>
       </text>
     </comment>
     <comment ref="Q3" authorId="0" shapeId="0">
       <text>
-        <t>Optional. Full registration/landing link starting with https://</t>
+        <t>Optional. 5 digits (or 5+4).</t>
       </text>
     </comment>
     <comment ref="R3" authorId="0" shapeId="0">
       <text>
+        <t>Optional. Full registration/landing link starting with https://</t>
+      </text>
+    </comment>
+    <comment ref="S3" authorId="0" shapeId="0">
+      <text>
         <t>Optional. One or more of: Ski, Splitboard, Motorized, Snowshoe. Separate multiple with commas.</t>
       </text>
     </comment>
-    <comment ref="S3" authorId="0" shapeId="0">
+    <comment ref="T3" authorId="0" shapeId="0">
       <text>
         <t>Optional. One or more of: For LGBTQ+, For Women, For Youth. Separate multiple with commas.</t>
       </text>
@@ -641,28 +646,29 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:S205"/>
+  <dimension ref="A1:T205"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="16" customWidth="1" min="4" max="4"/>
-    <col width="14" customWidth="1" min="5" max="5"/>
-    <col width="12" customWidth="1" min="6" max="6"/>
-    <col width="18" customWidth="1" min="7" max="7"/>
-    <col width="14" customWidth="1" min="8" max="8"/>
-    <col width="12" customWidth="1" min="9" max="9"/>
-    <col width="16" customWidth="1" min="10" max="10"/>
+    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="16" customWidth="1" min="5" max="5"/>
+    <col width="14" customWidth="1" min="6" max="6"/>
+    <col width="12" customWidth="1" min="7" max="7"/>
+    <col width="18" customWidth="1" min="8" max="8"/>
+    <col width="14" customWidth="1" min="9" max="9"/>
+    <col width="12" customWidth="1" min="10" max="10"/>
     <col width="16" customWidth="1" min="11" max="11"/>
-    <col width="24" customWidth="1" min="12" max="12"/>
-    <col width="26" customWidth="1" min="13" max="13"/>
-    <col width="18" customWidth="1" min="14" max="14"/>
-    <col width="10" customWidth="1" min="15" max="15"/>
-    <col width="12" customWidth="1" min="16" max="16"/>
-    <col width="34" customWidth="1" min="17" max="17"/>
-    <col width="26" customWidth="1" min="18" max="18"/>
+    <col width="16" customWidth="1" min="12" max="12"/>
+    <col width="24" customWidth="1" min="13" max="13"/>
+    <col width="26" customWidth="1" min="14" max="14"/>
+    <col width="18" customWidth="1" min="15" max="15"/>
+    <col width="10" customWidth="1" min="16" max="16"/>
+    <col width="12" customWidth="1" min="17" max="17"/>
+    <col width="34" customWidth="1" min="18" max="18"/>
     <col width="26" customWidth="1" min="19" max="19"/>
+    <col width="26" customWidth="1" min="20" max="20"/>
   </cols>
   <sheetData>
     <row r="1" ht="26" customHeight="1">
@@ -695,82 +701,87 @@
           <t>Description</t>
         </is>
       </c>
-      <c r="D3" s="3" t="inlineStr">
+      <c r="D3" s="4" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="E3" s="3" t="inlineStr">
         <is>
           <t>Course Type *</t>
         </is>
       </c>
-      <c r="E3" s="3" t="inlineStr">
+      <c r="F3" s="3" t="inlineStr">
         <is>
           <t>Start Date *</t>
         </is>
       </c>
-      <c r="F3" s="3" t="inlineStr">
+      <c r="G3" s="3" t="inlineStr">
         <is>
           <t>Start Time *</t>
         </is>
       </c>
-      <c r="G3" s="3" t="inlineStr">
+      <c r="H3" s="3" t="inlineStr">
         <is>
           <t>Time Zone *</t>
         </is>
       </c>
-      <c r="H3" s="4" t="inlineStr">
+      <c r="I3" s="4" t="inlineStr">
         <is>
           <t>End Date</t>
         </is>
       </c>
-      <c r="I3" s="4" t="inlineStr">
+      <c r="J3" s="4" t="inlineStr">
         <is>
           <t>End Time</t>
         </is>
       </c>
-      <c r="J3" s="4" t="inlineStr">
+      <c r="K3" s="4" t="inlineStr">
         <is>
           <t>Registration Deadline Date</t>
         </is>
       </c>
-      <c r="K3" s="4" t="inlineStr">
+      <c r="L3" s="4" t="inlineStr">
         <is>
           <t>Registration Deadline Time</t>
         </is>
       </c>
-      <c r="L3" s="3" t="inlineStr">
+      <c r="M3" s="3" t="inlineStr">
         <is>
           <t>Place Name *</t>
         </is>
       </c>
-      <c r="M3" s="4" t="inlineStr">
+      <c r="N3" s="4" t="inlineStr">
         <is>
           <t>Street Address</t>
         </is>
       </c>
-      <c r="N3" s="4" t="inlineStr">
+      <c r="O3" s="4" t="inlineStr">
         <is>
           <t>City</t>
         </is>
       </c>
-      <c r="O3" s="3" t="inlineStr">
+      <c r="P3" s="3" t="inlineStr">
         <is>
           <t>State *</t>
         </is>
       </c>
-      <c r="P3" s="4" t="inlineStr">
+      <c r="Q3" s="4" t="inlineStr">
         <is>
           <t>ZIP Code</t>
         </is>
       </c>
-      <c r="Q3" s="4" t="inlineStr">
+      <c r="R3" s="4" t="inlineStr">
         <is>
           <t>Course URL</t>
         </is>
       </c>
-      <c r="R3" s="4" t="inlineStr">
+      <c r="S3" s="4" t="inlineStr">
         <is>
           <t>Mode of Travel</t>
         </is>
       </c>
-      <c r="S3" s="4" t="inlineStr">
+      <c r="T3" s="4" t="inlineStr">
         <is>
           <t>Interest Groups</t>
         </is>
@@ -794,80 +805,85 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
+          <t>Northwest Avalanche Institute</t>
+        </is>
+      </c>
+      <c r="E4" s="5" t="inlineStr">
+        <is>
           <t>Rec 1</t>
         </is>
       </c>
-      <c r="E4" s="5" t="inlineStr">
+      <c r="F4" s="5" t="inlineStr">
         <is>
           <t>01/17/2026</t>
         </is>
       </c>
-      <c r="F4" s="5" t="inlineStr">
+      <c r="G4" s="5" t="inlineStr">
         <is>
           <t>8:30 AM</t>
         </is>
       </c>
-      <c r="G4" s="5" t="inlineStr">
+      <c r="H4" s="5" t="inlineStr">
         <is>
           <t>Pacific Time (PT)</t>
         </is>
       </c>
-      <c r="H4" s="5" t="inlineStr">
+      <c r="I4" s="5" t="inlineStr">
         <is>
           <t>01/18/2026</t>
         </is>
       </c>
-      <c r="I4" s="5" t="inlineStr">
+      <c r="J4" s="5" t="inlineStr">
         <is>
           <t>4:30 PM</t>
         </is>
       </c>
-      <c r="J4" s="5" t="inlineStr">
+      <c r="K4" s="5" t="inlineStr">
         <is>
           <t>01/10/2026</t>
         </is>
       </c>
-      <c r="K4" s="5" t="inlineStr">
+      <c r="L4" s="5" t="inlineStr">
         <is>
           <t>11:59 PM</t>
         </is>
       </c>
-      <c r="L4" s="5" t="inlineStr">
+      <c r="M4" s="5" t="inlineStr">
         <is>
           <t>Snoqualmie Pass Nordic Center</t>
         </is>
       </c>
-      <c r="M4" s="5" t="inlineStr">
+      <c r="N4" s="5" t="inlineStr">
         <is>
           <t>9000 Alpental Rd</t>
         </is>
       </c>
-      <c r="N4" s="5" t="inlineStr">
+      <c r="O4" s="5" t="inlineStr">
         <is>
           <t>Snoqualmie Pass</t>
         </is>
       </c>
-      <c r="O4" s="5" t="inlineStr">
+      <c r="P4" s="5" t="inlineStr">
         <is>
           <t>WA</t>
         </is>
       </c>
-      <c r="P4" s="5" t="inlineStr">
+      <c r="Q4" s="5" t="inlineStr">
         <is>
           <t>98068</t>
         </is>
       </c>
-      <c r="Q4" s="5" t="inlineStr">
+      <c r="R4" s="5" t="inlineStr">
         <is>
           <t>https://example.org/courses/rec-1</t>
         </is>
       </c>
-      <c r="R4" s="5" t="inlineStr">
+      <c r="S4" s="5" t="inlineStr">
         <is>
           <t>Ski, Splitboard</t>
         </is>
       </c>
-      <c r="S4" s="5" t="inlineStr">
+      <c r="T4" s="5" t="inlineStr">
         <is>
           <t>For Women</t>
         </is>
@@ -893,6 +909,7 @@
       <c r="Q5" s="6" t="n"/>
       <c r="R5" s="6" t="n"/>
       <c r="S5" s="6" t="n"/>
+      <c r="T5" s="6" t="n"/>
     </row>
     <row r="6">
       <c r="A6" s="6" t="n"/>
@@ -914,6 +931,7 @@
       <c r="Q6" s="6" t="n"/>
       <c r="R6" s="6" t="n"/>
       <c r="S6" s="6" t="n"/>
+      <c r="T6" s="6" t="n"/>
     </row>
     <row r="7">
       <c r="A7" s="6" t="n"/>
@@ -935,6 +953,7 @@
       <c r="Q7" s="6" t="n"/>
       <c r="R7" s="6" t="n"/>
       <c r="S7" s="6" t="n"/>
+      <c r="T7" s="6" t="n"/>
     </row>
     <row r="8">
       <c r="A8" s="6" t="n"/>
@@ -956,6 +975,7 @@
       <c r="Q8" s="6" t="n"/>
       <c r="R8" s="6" t="n"/>
       <c r="S8" s="6" t="n"/>
+      <c r="T8" s="6" t="n"/>
     </row>
     <row r="9">
       <c r="A9" s="6" t="n"/>
@@ -977,6 +997,7 @@
       <c r="Q9" s="6" t="n"/>
       <c r="R9" s="6" t="n"/>
       <c r="S9" s="6" t="n"/>
+      <c r="T9" s="6" t="n"/>
     </row>
     <row r="10">
       <c r="A10" s="6" t="n"/>
@@ -998,6 +1019,7 @@
       <c r="Q10" s="6" t="n"/>
       <c r="R10" s="6" t="n"/>
       <c r="S10" s="6" t="n"/>
+      <c r="T10" s="6" t="n"/>
     </row>
     <row r="11">
       <c r="A11" s="6" t="n"/>
@@ -1019,6 +1041,7 @@
       <c r="Q11" s="6" t="n"/>
       <c r="R11" s="6" t="n"/>
       <c r="S11" s="6" t="n"/>
+      <c r="T11" s="6" t="n"/>
     </row>
     <row r="12">
       <c r="A12" s="6" t="n"/>
@@ -1040,6 +1063,7 @@
       <c r="Q12" s="6" t="n"/>
       <c r="R12" s="6" t="n"/>
       <c r="S12" s="6" t="n"/>
+      <c r="T12" s="6" t="n"/>
     </row>
     <row r="13">
       <c r="A13" s="6" t="n"/>
@@ -1061,6 +1085,7 @@
       <c r="Q13" s="6" t="n"/>
       <c r="R13" s="6" t="n"/>
       <c r="S13" s="6" t="n"/>
+      <c r="T13" s="6" t="n"/>
     </row>
     <row r="14">
       <c r="A14" s="6" t="n"/>
@@ -1082,6 +1107,7 @@
       <c r="Q14" s="6" t="n"/>
       <c r="R14" s="6" t="n"/>
       <c r="S14" s="6" t="n"/>
+      <c r="T14" s="6" t="n"/>
     </row>
     <row r="15">
       <c r="A15" s="6" t="n"/>
@@ -1103,6 +1129,7 @@
       <c r="Q15" s="6" t="n"/>
       <c r="R15" s="6" t="n"/>
       <c r="S15" s="6" t="n"/>
+      <c r="T15" s="6" t="n"/>
     </row>
     <row r="16">
       <c r="A16" s="6" t="n"/>
@@ -1124,6 +1151,7 @@
       <c r="Q16" s="6" t="n"/>
       <c r="R16" s="6" t="n"/>
       <c r="S16" s="6" t="n"/>
+      <c r="T16" s="6" t="n"/>
     </row>
     <row r="17">
       <c r="A17" s="6" t="n"/>
@@ -1145,6 +1173,7 @@
       <c r="Q17" s="6" t="n"/>
       <c r="R17" s="6" t="n"/>
       <c r="S17" s="6" t="n"/>
+      <c r="T17" s="6" t="n"/>
     </row>
     <row r="18">
       <c r="A18" s="6" t="n"/>
@@ -1166,6 +1195,7 @@
       <c r="Q18" s="6" t="n"/>
       <c r="R18" s="6" t="n"/>
       <c r="S18" s="6" t="n"/>
+      <c r="T18" s="6" t="n"/>
     </row>
     <row r="19">
       <c r="A19" s="6" t="n"/>
@@ -1187,6 +1217,7 @@
       <c r="Q19" s="6" t="n"/>
       <c r="R19" s="6" t="n"/>
       <c r="S19" s="6" t="n"/>
+      <c r="T19" s="6" t="n"/>
     </row>
     <row r="20">
       <c r="A20" s="6" t="n"/>
@@ -1208,6 +1239,7 @@
       <c r="Q20" s="6" t="n"/>
       <c r="R20" s="6" t="n"/>
       <c r="S20" s="6" t="n"/>
+      <c r="T20" s="6" t="n"/>
     </row>
     <row r="21">
       <c r="A21" s="6" t="n"/>
@@ -1229,6 +1261,7 @@
       <c r="Q21" s="6" t="n"/>
       <c r="R21" s="6" t="n"/>
       <c r="S21" s="6" t="n"/>
+      <c r="T21" s="6" t="n"/>
     </row>
     <row r="22">
       <c r="A22" s="6" t="n"/>
@@ -1250,6 +1283,7 @@
       <c r="Q22" s="6" t="n"/>
       <c r="R22" s="6" t="n"/>
       <c r="S22" s="6" t="n"/>
+      <c r="T22" s="6" t="n"/>
     </row>
     <row r="23">
       <c r="A23" s="6" t="n"/>
@@ -1271,6 +1305,7 @@
       <c r="Q23" s="6" t="n"/>
       <c r="R23" s="6" t="n"/>
       <c r="S23" s="6" t="n"/>
+      <c r="T23" s="6" t="n"/>
     </row>
     <row r="24">
       <c r="A24" s="6" t="n"/>
@@ -1292,6 +1327,7 @@
       <c r="Q24" s="6" t="n"/>
       <c r="R24" s="6" t="n"/>
       <c r="S24" s="6" t="n"/>
+      <c r="T24" s="6" t="n"/>
     </row>
     <row r="25">
       <c r="A25" s="6" t="n"/>
@@ -1313,6 +1349,7 @@
       <c r="Q25" s="6" t="n"/>
       <c r="R25" s="6" t="n"/>
       <c r="S25" s="6" t="n"/>
+      <c r="T25" s="6" t="n"/>
     </row>
     <row r="26">
       <c r="A26" s="6" t="n"/>
@@ -1334,6 +1371,7 @@
       <c r="Q26" s="6" t="n"/>
       <c r="R26" s="6" t="n"/>
       <c r="S26" s="6" t="n"/>
+      <c r="T26" s="6" t="n"/>
     </row>
     <row r="27">
       <c r="A27" s="6" t="n"/>
@@ -1355,6 +1393,7 @@
       <c r="Q27" s="6" t="n"/>
       <c r="R27" s="6" t="n"/>
       <c r="S27" s="6" t="n"/>
+      <c r="T27" s="6" t="n"/>
     </row>
     <row r="28">
       <c r="A28" s="6" t="n"/>
@@ -1376,6 +1415,7 @@
       <c r="Q28" s="6" t="n"/>
       <c r="R28" s="6" t="n"/>
       <c r="S28" s="6" t="n"/>
+      <c r="T28" s="6" t="n"/>
     </row>
     <row r="29">
       <c r="A29" s="6" t="n"/>
@@ -1397,6 +1437,7 @@
       <c r="Q29" s="6" t="n"/>
       <c r="R29" s="6" t="n"/>
       <c r="S29" s="6" t="n"/>
+      <c r="T29" s="6" t="n"/>
     </row>
     <row r="30">
       <c r="A30" s="6" t="n"/>
@@ -1418,6 +1459,7 @@
       <c r="Q30" s="6" t="n"/>
       <c r="R30" s="6" t="n"/>
       <c r="S30" s="6" t="n"/>
+      <c r="T30" s="6" t="n"/>
     </row>
     <row r="31">
       <c r="A31" s="6" t="n"/>
@@ -1439,6 +1481,7 @@
       <c r="Q31" s="6" t="n"/>
       <c r="R31" s="6" t="n"/>
       <c r="S31" s="6" t="n"/>
+      <c r="T31" s="6" t="n"/>
     </row>
     <row r="32">
       <c r="A32" s="6" t="n"/>
@@ -1460,6 +1503,7 @@
       <c r="Q32" s="6" t="n"/>
       <c r="R32" s="6" t="n"/>
       <c r="S32" s="6" t="n"/>
+      <c r="T32" s="6" t="n"/>
     </row>
     <row r="33">
       <c r="A33" s="6" t="n"/>
@@ -1481,6 +1525,7 @@
       <c r="Q33" s="6" t="n"/>
       <c r="R33" s="6" t="n"/>
       <c r="S33" s="6" t="n"/>
+      <c r="T33" s="6" t="n"/>
     </row>
     <row r="34">
       <c r="A34" s="6" t="n"/>
@@ -1502,6 +1547,7 @@
       <c r="Q34" s="6" t="n"/>
       <c r="R34" s="6" t="n"/>
       <c r="S34" s="6" t="n"/>
+      <c r="T34" s="6" t="n"/>
     </row>
     <row r="35">
       <c r="A35" s="6" t="n"/>
@@ -1523,6 +1569,7 @@
       <c r="Q35" s="6" t="n"/>
       <c r="R35" s="6" t="n"/>
       <c r="S35" s="6" t="n"/>
+      <c r="T35" s="6" t="n"/>
     </row>
     <row r="36">
       <c r="A36" s="6" t="n"/>
@@ -1544,6 +1591,7 @@
       <c r="Q36" s="6" t="n"/>
       <c r="R36" s="6" t="n"/>
       <c r="S36" s="6" t="n"/>
+      <c r="T36" s="6" t="n"/>
     </row>
     <row r="37">
       <c r="A37" s="6" t="n"/>
@@ -1565,6 +1613,7 @@
       <c r="Q37" s="6" t="n"/>
       <c r="R37" s="6" t="n"/>
       <c r="S37" s="6" t="n"/>
+      <c r="T37" s="6" t="n"/>
     </row>
     <row r="38">
       <c r="A38" s="6" t="n"/>
@@ -1586,6 +1635,7 @@
       <c r="Q38" s="6" t="n"/>
       <c r="R38" s="6" t="n"/>
       <c r="S38" s="6" t="n"/>
+      <c r="T38" s="6" t="n"/>
     </row>
     <row r="39">
       <c r="A39" s="6" t="n"/>
@@ -1607,6 +1657,7 @@
       <c r="Q39" s="6" t="n"/>
       <c r="R39" s="6" t="n"/>
       <c r="S39" s="6" t="n"/>
+      <c r="T39" s="6" t="n"/>
     </row>
     <row r="40">
       <c r="A40" s="6" t="n"/>
@@ -1628,6 +1679,7 @@
       <c r="Q40" s="6" t="n"/>
       <c r="R40" s="6" t="n"/>
       <c r="S40" s="6" t="n"/>
+      <c r="T40" s="6" t="n"/>
     </row>
     <row r="41">
       <c r="A41" s="6" t="n"/>
@@ -1649,6 +1701,7 @@
       <c r="Q41" s="6" t="n"/>
       <c r="R41" s="6" t="n"/>
       <c r="S41" s="6" t="n"/>
+      <c r="T41" s="6" t="n"/>
     </row>
     <row r="42">
       <c r="A42" s="6" t="n"/>
@@ -1670,6 +1723,7 @@
       <c r="Q42" s="6" t="n"/>
       <c r="R42" s="6" t="n"/>
       <c r="S42" s="6" t="n"/>
+      <c r="T42" s="6" t="n"/>
     </row>
     <row r="43">
       <c r="A43" s="6" t="n"/>
@@ -1691,6 +1745,7 @@
       <c r="Q43" s="6" t="n"/>
       <c r="R43" s="6" t="n"/>
       <c r="S43" s="6" t="n"/>
+      <c r="T43" s="6" t="n"/>
     </row>
     <row r="44">
       <c r="A44" s="6" t="n"/>
@@ -1712,6 +1767,7 @@
       <c r="Q44" s="6" t="n"/>
       <c r="R44" s="6" t="n"/>
       <c r="S44" s="6" t="n"/>
+      <c r="T44" s="6" t="n"/>
     </row>
     <row r="45">
       <c r="A45" s="6" t="n"/>
@@ -1733,6 +1789,7 @@
       <c r="Q45" s="6" t="n"/>
       <c r="R45" s="6" t="n"/>
       <c r="S45" s="6" t="n"/>
+      <c r="T45" s="6" t="n"/>
     </row>
     <row r="46">
       <c r="A46" s="6" t="n"/>
@@ -1754,6 +1811,7 @@
       <c r="Q46" s="6" t="n"/>
       <c r="R46" s="6" t="n"/>
       <c r="S46" s="6" t="n"/>
+      <c r="T46" s="6" t="n"/>
     </row>
     <row r="47">
       <c r="A47" s="6" t="n"/>
@@ -1775,6 +1833,7 @@
       <c r="Q47" s="6" t="n"/>
       <c r="R47" s="6" t="n"/>
       <c r="S47" s="6" t="n"/>
+      <c r="T47" s="6" t="n"/>
     </row>
     <row r="48">
       <c r="A48" s="6" t="n"/>
@@ -1796,6 +1855,7 @@
       <c r="Q48" s="6" t="n"/>
       <c r="R48" s="6" t="n"/>
       <c r="S48" s="6" t="n"/>
+      <c r="T48" s="6" t="n"/>
     </row>
     <row r="49">
       <c r="A49" s="6" t="n"/>
@@ -1817,6 +1877,7 @@
       <c r="Q49" s="6" t="n"/>
       <c r="R49" s="6" t="n"/>
       <c r="S49" s="6" t="n"/>
+      <c r="T49" s="6" t="n"/>
     </row>
     <row r="50">
       <c r="A50" s="6" t="n"/>
@@ -1838,6 +1899,7 @@
       <c r="Q50" s="6" t="n"/>
       <c r="R50" s="6" t="n"/>
       <c r="S50" s="6" t="n"/>
+      <c r="T50" s="6" t="n"/>
     </row>
     <row r="51">
       <c r="A51" s="6" t="n"/>
@@ -1859,6 +1921,7 @@
       <c r="Q51" s="6" t="n"/>
       <c r="R51" s="6" t="n"/>
       <c r="S51" s="6" t="n"/>
+      <c r="T51" s="6" t="n"/>
     </row>
     <row r="52">
       <c r="A52" s="6" t="n"/>
@@ -1880,6 +1943,7 @@
       <c r="Q52" s="6" t="n"/>
       <c r="R52" s="6" t="n"/>
       <c r="S52" s="6" t="n"/>
+      <c r="T52" s="6" t="n"/>
     </row>
     <row r="53">
       <c r="A53" s="6" t="n"/>
@@ -1901,6 +1965,7 @@
       <c r="Q53" s="6" t="n"/>
       <c r="R53" s="6" t="n"/>
       <c r="S53" s="6" t="n"/>
+      <c r="T53" s="6" t="n"/>
     </row>
     <row r="54">
       <c r="A54" s="6" t="n"/>
@@ -1922,6 +1987,7 @@
       <c r="Q54" s="6" t="n"/>
       <c r="R54" s="6" t="n"/>
       <c r="S54" s="6" t="n"/>
+      <c r="T54" s="6" t="n"/>
     </row>
     <row r="55">
       <c r="A55" s="6" t="n"/>
@@ -1943,6 +2009,7 @@
       <c r="Q55" s="6" t="n"/>
       <c r="R55" s="6" t="n"/>
       <c r="S55" s="6" t="n"/>
+      <c r="T55" s="6" t="n"/>
     </row>
     <row r="56">
       <c r="A56" s="6" t="n"/>
@@ -1964,6 +2031,7 @@
       <c r="Q56" s="6" t="n"/>
       <c r="R56" s="6" t="n"/>
       <c r="S56" s="6" t="n"/>
+      <c r="T56" s="6" t="n"/>
     </row>
     <row r="57">
       <c r="A57" s="6" t="n"/>
@@ -1985,6 +2053,7 @@
       <c r="Q57" s="6" t="n"/>
       <c r="R57" s="6" t="n"/>
       <c r="S57" s="6" t="n"/>
+      <c r="T57" s="6" t="n"/>
     </row>
     <row r="58">
       <c r="A58" s="6" t="n"/>
@@ -2006,6 +2075,7 @@
       <c r="Q58" s="6" t="n"/>
       <c r="R58" s="6" t="n"/>
       <c r="S58" s="6" t="n"/>
+      <c r="T58" s="6" t="n"/>
     </row>
     <row r="59">
       <c r="A59" s="6" t="n"/>
@@ -2027,6 +2097,7 @@
       <c r="Q59" s="6" t="n"/>
       <c r="R59" s="6" t="n"/>
       <c r="S59" s="6" t="n"/>
+      <c r="T59" s="6" t="n"/>
     </row>
     <row r="60">
       <c r="A60" s="6" t="n"/>
@@ -2048,6 +2119,7 @@
       <c r="Q60" s="6" t="n"/>
       <c r="R60" s="6" t="n"/>
       <c r="S60" s="6" t="n"/>
+      <c r="T60" s="6" t="n"/>
     </row>
     <row r="61">
       <c r="A61" s="6" t="n"/>
@@ -2069,6 +2141,7 @@
       <c r="Q61" s="6" t="n"/>
       <c r="R61" s="6" t="n"/>
       <c r="S61" s="6" t="n"/>
+      <c r="T61" s="6" t="n"/>
     </row>
     <row r="62">
       <c r="A62" s="6" t="n"/>
@@ -2090,6 +2163,7 @@
       <c r="Q62" s="6" t="n"/>
       <c r="R62" s="6" t="n"/>
       <c r="S62" s="6" t="n"/>
+      <c r="T62" s="6" t="n"/>
     </row>
     <row r="63">
       <c r="A63" s="6" t="n"/>
@@ -2111,6 +2185,7 @@
       <c r="Q63" s="6" t="n"/>
       <c r="R63" s="6" t="n"/>
       <c r="S63" s="6" t="n"/>
+      <c r="T63" s="6" t="n"/>
     </row>
     <row r="64">
       <c r="A64" s="6" t="n"/>
@@ -2132,6 +2207,7 @@
       <c r="Q64" s="6" t="n"/>
       <c r="R64" s="6" t="n"/>
       <c r="S64" s="6" t="n"/>
+      <c r="T64" s="6" t="n"/>
     </row>
     <row r="65">
       <c r="A65" s="6" t="n"/>
@@ -2153,6 +2229,7 @@
       <c r="Q65" s="6" t="n"/>
       <c r="R65" s="6" t="n"/>
       <c r="S65" s="6" t="n"/>
+      <c r="T65" s="6" t="n"/>
     </row>
     <row r="66">
       <c r="A66" s="6" t="n"/>
@@ -2174,6 +2251,7 @@
       <c r="Q66" s="6" t="n"/>
       <c r="R66" s="6" t="n"/>
       <c r="S66" s="6" t="n"/>
+      <c r="T66" s="6" t="n"/>
     </row>
     <row r="67">
       <c r="A67" s="6" t="n"/>
@@ -2195,6 +2273,7 @@
       <c r="Q67" s="6" t="n"/>
       <c r="R67" s="6" t="n"/>
       <c r="S67" s="6" t="n"/>
+      <c r="T67" s="6" t="n"/>
     </row>
     <row r="68">
       <c r="A68" s="6" t="n"/>
@@ -2216,6 +2295,7 @@
       <c r="Q68" s="6" t="n"/>
       <c r="R68" s="6" t="n"/>
       <c r="S68" s="6" t="n"/>
+      <c r="T68" s="6" t="n"/>
     </row>
     <row r="69">
       <c r="A69" s="6" t="n"/>
@@ -2237,6 +2317,7 @@
       <c r="Q69" s="6" t="n"/>
       <c r="R69" s="6" t="n"/>
       <c r="S69" s="6" t="n"/>
+      <c r="T69" s="6" t="n"/>
     </row>
     <row r="70">
       <c r="A70" s="6" t="n"/>
@@ -2258,6 +2339,7 @@
       <c r="Q70" s="6" t="n"/>
       <c r="R70" s="6" t="n"/>
       <c r="S70" s="6" t="n"/>
+      <c r="T70" s="6" t="n"/>
     </row>
     <row r="71">
       <c r="A71" s="6" t="n"/>
@@ -2279,6 +2361,7 @@
       <c r="Q71" s="6" t="n"/>
       <c r="R71" s="6" t="n"/>
       <c r="S71" s="6" t="n"/>
+      <c r="T71" s="6" t="n"/>
     </row>
     <row r="72">
       <c r="A72" s="6" t="n"/>
@@ -2300,6 +2383,7 @@
       <c r="Q72" s="6" t="n"/>
       <c r="R72" s="6" t="n"/>
       <c r="S72" s="6" t="n"/>
+      <c r="T72" s="6" t="n"/>
     </row>
     <row r="73">
       <c r="A73" s="6" t="n"/>
@@ -2321,6 +2405,7 @@
       <c r="Q73" s="6" t="n"/>
       <c r="R73" s="6" t="n"/>
       <c r="S73" s="6" t="n"/>
+      <c r="T73" s="6" t="n"/>
     </row>
     <row r="74">
       <c r="A74" s="6" t="n"/>
@@ -2342,6 +2427,7 @@
       <c r="Q74" s="6" t="n"/>
       <c r="R74" s="6" t="n"/>
       <c r="S74" s="6" t="n"/>
+      <c r="T74" s="6" t="n"/>
     </row>
     <row r="75">
       <c r="A75" s="6" t="n"/>
@@ -2363,6 +2449,7 @@
       <c r="Q75" s="6" t="n"/>
       <c r="R75" s="6" t="n"/>
       <c r="S75" s="6" t="n"/>
+      <c r="T75" s="6" t="n"/>
     </row>
     <row r="76">
       <c r="A76" s="6" t="n"/>
@@ -2384,6 +2471,7 @@
       <c r="Q76" s="6" t="n"/>
       <c r="R76" s="6" t="n"/>
       <c r="S76" s="6" t="n"/>
+      <c r="T76" s="6" t="n"/>
     </row>
     <row r="77">
       <c r="A77" s="6" t="n"/>
@@ -2405,6 +2493,7 @@
       <c r="Q77" s="6" t="n"/>
       <c r="R77" s="6" t="n"/>
       <c r="S77" s="6" t="n"/>
+      <c r="T77" s="6" t="n"/>
     </row>
     <row r="78">
       <c r="A78" s="6" t="n"/>
@@ -2426,6 +2515,7 @@
       <c r="Q78" s="6" t="n"/>
       <c r="R78" s="6" t="n"/>
       <c r="S78" s="6" t="n"/>
+      <c r="T78" s="6" t="n"/>
     </row>
     <row r="79">
       <c r="A79" s="6" t="n"/>
@@ -2447,6 +2537,7 @@
       <c r="Q79" s="6" t="n"/>
       <c r="R79" s="6" t="n"/>
       <c r="S79" s="6" t="n"/>
+      <c r="T79" s="6" t="n"/>
     </row>
     <row r="80">
       <c r="A80" s="6" t="n"/>
@@ -2468,6 +2559,7 @@
       <c r="Q80" s="6" t="n"/>
       <c r="R80" s="6" t="n"/>
       <c r="S80" s="6" t="n"/>
+      <c r="T80" s="6" t="n"/>
     </row>
     <row r="81">
       <c r="A81" s="6" t="n"/>
@@ -2489,6 +2581,7 @@
       <c r="Q81" s="6" t="n"/>
       <c r="R81" s="6" t="n"/>
       <c r="S81" s="6" t="n"/>
+      <c r="T81" s="6" t="n"/>
     </row>
     <row r="82">
       <c r="A82" s="6" t="n"/>
@@ -2510,6 +2603,7 @@
       <c r="Q82" s="6" t="n"/>
       <c r="R82" s="6" t="n"/>
       <c r="S82" s="6" t="n"/>
+      <c r="T82" s="6" t="n"/>
     </row>
     <row r="83">
       <c r="A83" s="6" t="n"/>
@@ -2531,6 +2625,7 @@
       <c r="Q83" s="6" t="n"/>
       <c r="R83" s="6" t="n"/>
       <c r="S83" s="6" t="n"/>
+      <c r="T83" s="6" t="n"/>
     </row>
     <row r="84">
       <c r="A84" s="6" t="n"/>
@@ -2552,6 +2647,7 @@
       <c r="Q84" s="6" t="n"/>
       <c r="R84" s="6" t="n"/>
       <c r="S84" s="6" t="n"/>
+      <c r="T84" s="6" t="n"/>
     </row>
     <row r="85">
       <c r="A85" s="6" t="n"/>
@@ -2573,6 +2669,7 @@
       <c r="Q85" s="6" t="n"/>
       <c r="R85" s="6" t="n"/>
       <c r="S85" s="6" t="n"/>
+      <c r="T85" s="6" t="n"/>
     </row>
     <row r="86">
       <c r="A86" s="6" t="n"/>
@@ -2594,6 +2691,7 @@
       <c r="Q86" s="6" t="n"/>
       <c r="R86" s="6" t="n"/>
       <c r="S86" s="6" t="n"/>
+      <c r="T86" s="6" t="n"/>
     </row>
     <row r="87">
       <c r="A87" s="6" t="n"/>
@@ -2615,6 +2713,7 @@
       <c r="Q87" s="6" t="n"/>
       <c r="R87" s="6" t="n"/>
       <c r="S87" s="6" t="n"/>
+      <c r="T87" s="6" t="n"/>
     </row>
     <row r="88">
       <c r="A88" s="6" t="n"/>
@@ -2636,6 +2735,7 @@
       <c r="Q88" s="6" t="n"/>
       <c r="R88" s="6" t="n"/>
       <c r="S88" s="6" t="n"/>
+      <c r="T88" s="6" t="n"/>
     </row>
     <row r="89">
       <c r="A89" s="6" t="n"/>
@@ -2657,6 +2757,7 @@
       <c r="Q89" s="6" t="n"/>
       <c r="R89" s="6" t="n"/>
       <c r="S89" s="6" t="n"/>
+      <c r="T89" s="6" t="n"/>
     </row>
     <row r="90">
       <c r="A90" s="6" t="n"/>
@@ -2678,6 +2779,7 @@
       <c r="Q90" s="6" t="n"/>
       <c r="R90" s="6" t="n"/>
       <c r="S90" s="6" t="n"/>
+      <c r="T90" s="6" t="n"/>
     </row>
     <row r="91">
       <c r="A91" s="6" t="n"/>
@@ -2699,6 +2801,7 @@
       <c r="Q91" s="6" t="n"/>
       <c r="R91" s="6" t="n"/>
       <c r="S91" s="6" t="n"/>
+      <c r="T91" s="6" t="n"/>
     </row>
     <row r="92">
       <c r="A92" s="6" t="n"/>
@@ -2720,6 +2823,7 @@
       <c r="Q92" s="6" t="n"/>
       <c r="R92" s="6" t="n"/>
       <c r="S92" s="6" t="n"/>
+      <c r="T92" s="6" t="n"/>
     </row>
     <row r="93">
       <c r="A93" s="6" t="n"/>
@@ -2741,6 +2845,7 @@
       <c r="Q93" s="6" t="n"/>
       <c r="R93" s="6" t="n"/>
       <c r="S93" s="6" t="n"/>
+      <c r="T93" s="6" t="n"/>
     </row>
     <row r="94">
       <c r="A94" s="6" t="n"/>
@@ -2762,6 +2867,7 @@
       <c r="Q94" s="6" t="n"/>
       <c r="R94" s="6" t="n"/>
       <c r="S94" s="6" t="n"/>
+      <c r="T94" s="6" t="n"/>
     </row>
     <row r="95">
       <c r="A95" s="6" t="n"/>
@@ -2783,6 +2889,7 @@
       <c r="Q95" s="6" t="n"/>
       <c r="R95" s="6" t="n"/>
       <c r="S95" s="6" t="n"/>
+      <c r="T95" s="6" t="n"/>
     </row>
     <row r="96">
       <c r="A96" s="6" t="n"/>
@@ -2804,6 +2911,7 @@
       <c r="Q96" s="6" t="n"/>
       <c r="R96" s="6" t="n"/>
       <c r="S96" s="6" t="n"/>
+      <c r="T96" s="6" t="n"/>
     </row>
     <row r="97">
       <c r="A97" s="6" t="n"/>
@@ -2825,6 +2933,7 @@
       <c r="Q97" s="6" t="n"/>
       <c r="R97" s="6" t="n"/>
       <c r="S97" s="6" t="n"/>
+      <c r="T97" s="6" t="n"/>
     </row>
     <row r="98">
       <c r="A98" s="6" t="n"/>
@@ -2846,6 +2955,7 @@
       <c r="Q98" s="6" t="n"/>
       <c r="R98" s="6" t="n"/>
       <c r="S98" s="6" t="n"/>
+      <c r="T98" s="6" t="n"/>
     </row>
     <row r="99">
       <c r="A99" s="6" t="n"/>
@@ -2867,6 +2977,7 @@
       <c r="Q99" s="6" t="n"/>
       <c r="R99" s="6" t="n"/>
       <c r="S99" s="6" t="n"/>
+      <c r="T99" s="6" t="n"/>
     </row>
     <row r="100">
       <c r="A100" s="6" t="n"/>
@@ -2888,6 +2999,7 @@
       <c r="Q100" s="6" t="n"/>
       <c r="R100" s="6" t="n"/>
       <c r="S100" s="6" t="n"/>
+      <c r="T100" s="6" t="n"/>
     </row>
     <row r="101">
       <c r="A101" s="6" t="n"/>
@@ -2909,6 +3021,7 @@
       <c r="Q101" s="6" t="n"/>
       <c r="R101" s="6" t="n"/>
       <c r="S101" s="6" t="n"/>
+      <c r="T101" s="6" t="n"/>
     </row>
     <row r="102">
       <c r="A102" s="6" t="n"/>
@@ -2930,6 +3043,7 @@
       <c r="Q102" s="6" t="n"/>
       <c r="R102" s="6" t="n"/>
       <c r="S102" s="6" t="n"/>
+      <c r="T102" s="6" t="n"/>
     </row>
     <row r="103">
       <c r="A103" s="6" t="n"/>
@@ -2951,6 +3065,7 @@
       <c r="Q103" s="6" t="n"/>
       <c r="R103" s="6" t="n"/>
       <c r="S103" s="6" t="n"/>
+      <c r="T103" s="6" t="n"/>
     </row>
     <row r="104">
       <c r="A104" s="6" t="n"/>
@@ -2972,6 +3087,7 @@
       <c r="Q104" s="6" t="n"/>
       <c r="R104" s="6" t="n"/>
       <c r="S104" s="6" t="n"/>
+      <c r="T104" s="6" t="n"/>
     </row>
     <row r="105">
       <c r="A105" s="6" t="n"/>
@@ -2993,6 +3109,7 @@
       <c r="Q105" s="6" t="n"/>
       <c r="R105" s="6" t="n"/>
       <c r="S105" s="6" t="n"/>
+      <c r="T105" s="6" t="n"/>
     </row>
     <row r="106">
       <c r="A106" s="6" t="n"/>
@@ -3014,6 +3131,7 @@
       <c r="Q106" s="6" t="n"/>
       <c r="R106" s="6" t="n"/>
       <c r="S106" s="6" t="n"/>
+      <c r="T106" s="6" t="n"/>
     </row>
     <row r="107">
       <c r="A107" s="6" t="n"/>
@@ -3035,6 +3153,7 @@
       <c r="Q107" s="6" t="n"/>
       <c r="R107" s="6" t="n"/>
       <c r="S107" s="6" t="n"/>
+      <c r="T107" s="6" t="n"/>
     </row>
     <row r="108">
       <c r="A108" s="6" t="n"/>
@@ -3056,6 +3175,7 @@
       <c r="Q108" s="6" t="n"/>
       <c r="R108" s="6" t="n"/>
       <c r="S108" s="6" t="n"/>
+      <c r="T108" s="6" t="n"/>
     </row>
     <row r="109">
       <c r="A109" s="6" t="n"/>
@@ -3077,6 +3197,7 @@
       <c r="Q109" s="6" t="n"/>
       <c r="R109" s="6" t="n"/>
       <c r="S109" s="6" t="n"/>
+      <c r="T109" s="6" t="n"/>
     </row>
     <row r="110">
       <c r="A110" s="6" t="n"/>
@@ -3098,6 +3219,7 @@
       <c r="Q110" s="6" t="n"/>
       <c r="R110" s="6" t="n"/>
       <c r="S110" s="6" t="n"/>
+      <c r="T110" s="6" t="n"/>
     </row>
     <row r="111">
       <c r="A111" s="6" t="n"/>
@@ -3119,6 +3241,7 @@
       <c r="Q111" s="6" t="n"/>
       <c r="R111" s="6" t="n"/>
       <c r="S111" s="6" t="n"/>
+      <c r="T111" s="6" t="n"/>
     </row>
     <row r="112">
       <c r="A112" s="6" t="n"/>
@@ -3140,6 +3263,7 @@
       <c r="Q112" s="6" t="n"/>
       <c r="R112" s="6" t="n"/>
       <c r="S112" s="6" t="n"/>
+      <c r="T112" s="6" t="n"/>
     </row>
     <row r="113">
       <c r="A113" s="6" t="n"/>
@@ -3161,6 +3285,7 @@
       <c r="Q113" s="6" t="n"/>
       <c r="R113" s="6" t="n"/>
       <c r="S113" s="6" t="n"/>
+      <c r="T113" s="6" t="n"/>
     </row>
     <row r="114">
       <c r="A114" s="6" t="n"/>
@@ -3182,6 +3307,7 @@
       <c r="Q114" s="6" t="n"/>
       <c r="R114" s="6" t="n"/>
       <c r="S114" s="6" t="n"/>
+      <c r="T114" s="6" t="n"/>
     </row>
     <row r="115">
       <c r="A115" s="6" t="n"/>
@@ -3203,6 +3329,7 @@
       <c r="Q115" s="6" t="n"/>
       <c r="R115" s="6" t="n"/>
       <c r="S115" s="6" t="n"/>
+      <c r="T115" s="6" t="n"/>
     </row>
     <row r="116">
       <c r="A116" s="6" t="n"/>
@@ -3224,6 +3351,7 @@
       <c r="Q116" s="6" t="n"/>
       <c r="R116" s="6" t="n"/>
       <c r="S116" s="6" t="n"/>
+      <c r="T116" s="6" t="n"/>
     </row>
     <row r="117">
       <c r="A117" s="6" t="n"/>
@@ -3245,6 +3373,7 @@
       <c r="Q117" s="6" t="n"/>
       <c r="R117" s="6" t="n"/>
       <c r="S117" s="6" t="n"/>
+      <c r="T117" s="6" t="n"/>
     </row>
     <row r="118">
       <c r="A118" s="6" t="n"/>
@@ -3266,6 +3395,7 @@
       <c r="Q118" s="6" t="n"/>
       <c r="R118" s="6" t="n"/>
       <c r="S118" s="6" t="n"/>
+      <c r="T118" s="6" t="n"/>
     </row>
     <row r="119">
       <c r="A119" s="6" t="n"/>
@@ -3287,6 +3417,7 @@
       <c r="Q119" s="6" t="n"/>
       <c r="R119" s="6" t="n"/>
       <c r="S119" s="6" t="n"/>
+      <c r="T119" s="6" t="n"/>
     </row>
     <row r="120">
       <c r="A120" s="6" t="n"/>
@@ -3308,6 +3439,7 @@
       <c r="Q120" s="6" t="n"/>
       <c r="R120" s="6" t="n"/>
       <c r="S120" s="6" t="n"/>
+      <c r="T120" s="6" t="n"/>
     </row>
     <row r="121">
       <c r="A121" s="6" t="n"/>
@@ -3329,6 +3461,7 @@
       <c r="Q121" s="6" t="n"/>
       <c r="R121" s="6" t="n"/>
       <c r="S121" s="6" t="n"/>
+      <c r="T121" s="6" t="n"/>
     </row>
     <row r="122">
       <c r="A122" s="6" t="n"/>
@@ -3350,6 +3483,7 @@
       <c r="Q122" s="6" t="n"/>
       <c r="R122" s="6" t="n"/>
       <c r="S122" s="6" t="n"/>
+      <c r="T122" s="6" t="n"/>
     </row>
     <row r="123">
       <c r="A123" s="6" t="n"/>
@@ -3371,6 +3505,7 @@
       <c r="Q123" s="6" t="n"/>
       <c r="R123" s="6" t="n"/>
       <c r="S123" s="6" t="n"/>
+      <c r="T123" s="6" t="n"/>
     </row>
     <row r="124">
       <c r="A124" s="6" t="n"/>
@@ -3392,6 +3527,7 @@
       <c r="Q124" s="6" t="n"/>
       <c r="R124" s="6" t="n"/>
       <c r="S124" s="6" t="n"/>
+      <c r="T124" s="6" t="n"/>
     </row>
     <row r="125">
       <c r="A125" s="6" t="n"/>
@@ -3413,6 +3549,7 @@
       <c r="Q125" s="6" t="n"/>
       <c r="R125" s="6" t="n"/>
       <c r="S125" s="6" t="n"/>
+      <c r="T125" s="6" t="n"/>
     </row>
     <row r="126">
       <c r="A126" s="6" t="n"/>
@@ -3434,6 +3571,7 @@
       <c r="Q126" s="6" t="n"/>
       <c r="R126" s="6" t="n"/>
       <c r="S126" s="6" t="n"/>
+      <c r="T126" s="6" t="n"/>
     </row>
     <row r="127">
       <c r="A127" s="6" t="n"/>
@@ -3455,6 +3593,7 @@
       <c r="Q127" s="6" t="n"/>
       <c r="R127" s="6" t="n"/>
       <c r="S127" s="6" t="n"/>
+      <c r="T127" s="6" t="n"/>
     </row>
     <row r="128">
       <c r="A128" s="6" t="n"/>
@@ -3476,6 +3615,7 @@
       <c r="Q128" s="6" t="n"/>
       <c r="R128" s="6" t="n"/>
       <c r="S128" s="6" t="n"/>
+      <c r="T128" s="6" t="n"/>
     </row>
     <row r="129">
       <c r="A129" s="6" t="n"/>
@@ -3497,6 +3637,7 @@
       <c r="Q129" s="6" t="n"/>
       <c r="R129" s="6" t="n"/>
       <c r="S129" s="6" t="n"/>
+      <c r="T129" s="6" t="n"/>
     </row>
     <row r="130">
       <c r="A130" s="6" t="n"/>
@@ -3518,6 +3659,7 @@
       <c r="Q130" s="6" t="n"/>
       <c r="R130" s="6" t="n"/>
       <c r="S130" s="6" t="n"/>
+      <c r="T130" s="6" t="n"/>
     </row>
     <row r="131">
       <c r="A131" s="6" t="n"/>
@@ -3539,6 +3681,7 @@
       <c r="Q131" s="6" t="n"/>
       <c r="R131" s="6" t="n"/>
       <c r="S131" s="6" t="n"/>
+      <c r="T131" s="6" t="n"/>
     </row>
     <row r="132">
       <c r="A132" s="6" t="n"/>
@@ -3560,6 +3703,7 @@
       <c r="Q132" s="6" t="n"/>
       <c r="R132" s="6" t="n"/>
       <c r="S132" s="6" t="n"/>
+      <c r="T132" s="6" t="n"/>
     </row>
     <row r="133">
       <c r="A133" s="6" t="n"/>
@@ -3581,6 +3725,7 @@
       <c r="Q133" s="6" t="n"/>
       <c r="R133" s="6" t="n"/>
       <c r="S133" s="6" t="n"/>
+      <c r="T133" s="6" t="n"/>
     </row>
     <row r="134">
       <c r="A134" s="6" t="n"/>
@@ -3602,6 +3747,7 @@
       <c r="Q134" s="6" t="n"/>
       <c r="R134" s="6" t="n"/>
       <c r="S134" s="6" t="n"/>
+      <c r="T134" s="6" t="n"/>
     </row>
     <row r="135">
       <c r="A135" s="6" t="n"/>
@@ -3623,6 +3769,7 @@
       <c r="Q135" s="6" t="n"/>
       <c r="R135" s="6" t="n"/>
       <c r="S135" s="6" t="n"/>
+      <c r="T135" s="6" t="n"/>
     </row>
     <row r="136">
       <c r="A136" s="6" t="n"/>
@@ -3644,6 +3791,7 @@
       <c r="Q136" s="6" t="n"/>
       <c r="R136" s="6" t="n"/>
       <c r="S136" s="6" t="n"/>
+      <c r="T136" s="6" t="n"/>
     </row>
     <row r="137">
       <c r="A137" s="6" t="n"/>
@@ -3665,6 +3813,7 @@
       <c r="Q137" s="6" t="n"/>
       <c r="R137" s="6" t="n"/>
       <c r="S137" s="6" t="n"/>
+      <c r="T137" s="6" t="n"/>
     </row>
     <row r="138">
       <c r="A138" s="6" t="n"/>
@@ -3686,6 +3835,7 @@
       <c r="Q138" s="6" t="n"/>
       <c r="R138" s="6" t="n"/>
       <c r="S138" s="6" t="n"/>
+      <c r="T138" s="6" t="n"/>
     </row>
     <row r="139">
       <c r="A139" s="6" t="n"/>
@@ -3707,6 +3857,7 @@
       <c r="Q139" s="6" t="n"/>
       <c r="R139" s="6" t="n"/>
       <c r="S139" s="6" t="n"/>
+      <c r="T139" s="6" t="n"/>
     </row>
     <row r="140">
       <c r="A140" s="6" t="n"/>
@@ -3728,6 +3879,7 @@
       <c r="Q140" s="6" t="n"/>
       <c r="R140" s="6" t="n"/>
       <c r="S140" s="6" t="n"/>
+      <c r="T140" s="6" t="n"/>
     </row>
     <row r="141">
       <c r="A141" s="6" t="n"/>
@@ -3749,6 +3901,7 @@
       <c r="Q141" s="6" t="n"/>
       <c r="R141" s="6" t="n"/>
       <c r="S141" s="6" t="n"/>
+      <c r="T141" s="6" t="n"/>
     </row>
     <row r="142">
       <c r="A142" s="6" t="n"/>
@@ -3770,6 +3923,7 @@
       <c r="Q142" s="6" t="n"/>
       <c r="R142" s="6" t="n"/>
       <c r="S142" s="6" t="n"/>
+      <c r="T142" s="6" t="n"/>
     </row>
     <row r="143">
       <c r="A143" s="6" t="n"/>
@@ -3791,6 +3945,7 @@
       <c r="Q143" s="6" t="n"/>
       <c r="R143" s="6" t="n"/>
       <c r="S143" s="6" t="n"/>
+      <c r="T143" s="6" t="n"/>
     </row>
     <row r="144">
       <c r="A144" s="6" t="n"/>
@@ -3812,6 +3967,7 @@
       <c r="Q144" s="6" t="n"/>
       <c r="R144" s="6" t="n"/>
       <c r="S144" s="6" t="n"/>
+      <c r="T144" s="6" t="n"/>
     </row>
     <row r="145">
       <c r="A145" s="6" t="n"/>
@@ -3833,6 +3989,7 @@
       <c r="Q145" s="6" t="n"/>
       <c r="R145" s="6" t="n"/>
       <c r="S145" s="6" t="n"/>
+      <c r="T145" s="6" t="n"/>
     </row>
     <row r="146">
       <c r="A146" s="6" t="n"/>
@@ -3854,6 +4011,7 @@
       <c r="Q146" s="6" t="n"/>
       <c r="R146" s="6" t="n"/>
       <c r="S146" s="6" t="n"/>
+      <c r="T146" s="6" t="n"/>
     </row>
     <row r="147">
       <c r="A147" s="6" t="n"/>
@@ -3875,6 +4033,7 @@
       <c r="Q147" s="6" t="n"/>
       <c r="R147" s="6" t="n"/>
       <c r="S147" s="6" t="n"/>
+      <c r="T147" s="6" t="n"/>
     </row>
     <row r="148">
       <c r="A148" s="6" t="n"/>
@@ -3896,6 +4055,7 @@
       <c r="Q148" s="6" t="n"/>
       <c r="R148" s="6" t="n"/>
       <c r="S148" s="6" t="n"/>
+      <c r="T148" s="6" t="n"/>
     </row>
     <row r="149">
       <c r="A149" s="6" t="n"/>
@@ -3917,6 +4077,7 @@
       <c r="Q149" s="6" t="n"/>
       <c r="R149" s="6" t="n"/>
       <c r="S149" s="6" t="n"/>
+      <c r="T149" s="6" t="n"/>
     </row>
     <row r="150">
       <c r="A150" s="6" t="n"/>
@@ -3938,6 +4099,7 @@
       <c r="Q150" s="6" t="n"/>
       <c r="R150" s="6" t="n"/>
       <c r="S150" s="6" t="n"/>
+      <c r="T150" s="6" t="n"/>
     </row>
     <row r="151">
       <c r="A151" s="6" t="n"/>
@@ -3959,6 +4121,7 @@
       <c r="Q151" s="6" t="n"/>
       <c r="R151" s="6" t="n"/>
       <c r="S151" s="6" t="n"/>
+      <c r="T151" s="6" t="n"/>
     </row>
     <row r="152">
       <c r="A152" s="6" t="n"/>
@@ -3980,6 +4143,7 @@
       <c r="Q152" s="6" t="n"/>
       <c r="R152" s="6" t="n"/>
       <c r="S152" s="6" t="n"/>
+      <c r="T152" s="6" t="n"/>
     </row>
     <row r="153">
       <c r="A153" s="6" t="n"/>
@@ -4001,6 +4165,7 @@
       <c r="Q153" s="6" t="n"/>
       <c r="R153" s="6" t="n"/>
       <c r="S153" s="6" t="n"/>
+      <c r="T153" s="6" t="n"/>
     </row>
     <row r="154">
       <c r="A154" s="6" t="n"/>
@@ -4022,6 +4187,7 @@
       <c r="Q154" s="6" t="n"/>
       <c r="R154" s="6" t="n"/>
       <c r="S154" s="6" t="n"/>
+      <c r="T154" s="6" t="n"/>
     </row>
     <row r="155">
       <c r="A155" s="6" t="n"/>
@@ -4043,6 +4209,7 @@
       <c r="Q155" s="6" t="n"/>
       <c r="R155" s="6" t="n"/>
       <c r="S155" s="6" t="n"/>
+      <c r="T155" s="6" t="n"/>
     </row>
     <row r="156">
       <c r="A156" s="6" t="n"/>
@@ -4064,6 +4231,7 @@
       <c r="Q156" s="6" t="n"/>
       <c r="R156" s="6" t="n"/>
       <c r="S156" s="6" t="n"/>
+      <c r="T156" s="6" t="n"/>
     </row>
     <row r="157">
       <c r="A157" s="6" t="n"/>
@@ -4085,6 +4253,7 @@
       <c r="Q157" s="6" t="n"/>
       <c r="R157" s="6" t="n"/>
       <c r="S157" s="6" t="n"/>
+      <c r="T157" s="6" t="n"/>
     </row>
     <row r="158">
       <c r="A158" s="6" t="n"/>
@@ -4106,6 +4275,7 @@
       <c r="Q158" s="6" t="n"/>
       <c r="R158" s="6" t="n"/>
       <c r="S158" s="6" t="n"/>
+      <c r="T158" s="6" t="n"/>
     </row>
     <row r="159">
       <c r="A159" s="6" t="n"/>
@@ -4127,6 +4297,7 @@
       <c r="Q159" s="6" t="n"/>
       <c r="R159" s="6" t="n"/>
       <c r="S159" s="6" t="n"/>
+      <c r="T159" s="6" t="n"/>
     </row>
     <row r="160">
       <c r="A160" s="6" t="n"/>
@@ -4148,6 +4319,7 @@
       <c r="Q160" s="6" t="n"/>
       <c r="R160" s="6" t="n"/>
       <c r="S160" s="6" t="n"/>
+      <c r="T160" s="6" t="n"/>
     </row>
     <row r="161">
       <c r="A161" s="6" t="n"/>
@@ -4169,6 +4341,7 @@
       <c r="Q161" s="6" t="n"/>
       <c r="R161" s="6" t="n"/>
       <c r="S161" s="6" t="n"/>
+      <c r="T161" s="6" t="n"/>
     </row>
     <row r="162">
       <c r="A162" s="6" t="n"/>
@@ -4190,6 +4363,7 @@
       <c r="Q162" s="6" t="n"/>
       <c r="R162" s="6" t="n"/>
       <c r="S162" s="6" t="n"/>
+      <c r="T162" s="6" t="n"/>
     </row>
     <row r="163">
       <c r="A163" s="6" t="n"/>
@@ -4211,6 +4385,7 @@
       <c r="Q163" s="6" t="n"/>
       <c r="R163" s="6" t="n"/>
       <c r="S163" s="6" t="n"/>
+      <c r="T163" s="6" t="n"/>
     </row>
     <row r="164">
       <c r="A164" s="6" t="n"/>
@@ -4232,6 +4407,7 @@
       <c r="Q164" s="6" t="n"/>
       <c r="R164" s="6" t="n"/>
       <c r="S164" s="6" t="n"/>
+      <c r="T164" s="6" t="n"/>
     </row>
     <row r="165">
       <c r="A165" s="6" t="n"/>
@@ -4253,6 +4429,7 @@
       <c r="Q165" s="6" t="n"/>
       <c r="R165" s="6" t="n"/>
       <c r="S165" s="6" t="n"/>
+      <c r="T165" s="6" t="n"/>
     </row>
     <row r="166">
       <c r="A166" s="6" t="n"/>
@@ -4274,6 +4451,7 @@
       <c r="Q166" s="6" t="n"/>
       <c r="R166" s="6" t="n"/>
       <c r="S166" s="6" t="n"/>
+      <c r="T166" s="6" t="n"/>
     </row>
     <row r="167">
       <c r="A167" s="6" t="n"/>
@@ -4295,6 +4473,7 @@
       <c r="Q167" s="6" t="n"/>
       <c r="R167" s="6" t="n"/>
       <c r="S167" s="6" t="n"/>
+      <c r="T167" s="6" t="n"/>
     </row>
     <row r="168">
       <c r="A168" s="6" t="n"/>
@@ -4316,6 +4495,7 @@
       <c r="Q168" s="6" t="n"/>
       <c r="R168" s="6" t="n"/>
       <c r="S168" s="6" t="n"/>
+      <c r="T168" s="6" t="n"/>
     </row>
     <row r="169">
       <c r="A169" s="6" t="n"/>
@@ -4337,6 +4517,7 @@
       <c r="Q169" s="6" t="n"/>
       <c r="R169" s="6" t="n"/>
       <c r="S169" s="6" t="n"/>
+      <c r="T169" s="6" t="n"/>
     </row>
     <row r="170">
       <c r="A170" s="6" t="n"/>
@@ -4358,6 +4539,7 @@
       <c r="Q170" s="6" t="n"/>
       <c r="R170" s="6" t="n"/>
       <c r="S170" s="6" t="n"/>
+      <c r="T170" s="6" t="n"/>
     </row>
     <row r="171">
       <c r="A171" s="6" t="n"/>
@@ -4379,6 +4561,7 @@
       <c r="Q171" s="6" t="n"/>
       <c r="R171" s="6" t="n"/>
       <c r="S171" s="6" t="n"/>
+      <c r="T171" s="6" t="n"/>
     </row>
     <row r="172">
       <c r="A172" s="6" t="n"/>
@@ -4400,6 +4583,7 @@
       <c r="Q172" s="6" t="n"/>
       <c r="R172" s="6" t="n"/>
       <c r="S172" s="6" t="n"/>
+      <c r="T172" s="6" t="n"/>
     </row>
     <row r="173">
       <c r="A173" s="6" t="n"/>
@@ -4421,6 +4605,7 @@
       <c r="Q173" s="6" t="n"/>
       <c r="R173" s="6" t="n"/>
       <c r="S173" s="6" t="n"/>
+      <c r="T173" s="6" t="n"/>
     </row>
     <row r="174">
       <c r="A174" s="6" t="n"/>
@@ -4442,6 +4627,7 @@
       <c r="Q174" s="6" t="n"/>
       <c r="R174" s="6" t="n"/>
       <c r="S174" s="6" t="n"/>
+      <c r="T174" s="6" t="n"/>
     </row>
     <row r="175">
       <c r="A175" s="6" t="n"/>
@@ -4463,6 +4649,7 @@
       <c r="Q175" s="6" t="n"/>
       <c r="R175" s="6" t="n"/>
       <c r="S175" s="6" t="n"/>
+      <c r="T175" s="6" t="n"/>
     </row>
     <row r="176">
       <c r="A176" s="6" t="n"/>
@@ -4484,6 +4671,7 @@
       <c r="Q176" s="6" t="n"/>
       <c r="R176" s="6" t="n"/>
       <c r="S176" s="6" t="n"/>
+      <c r="T176" s="6" t="n"/>
     </row>
     <row r="177">
       <c r="A177" s="6" t="n"/>
@@ -4505,6 +4693,7 @@
       <c r="Q177" s="6" t="n"/>
       <c r="R177" s="6" t="n"/>
       <c r="S177" s="6" t="n"/>
+      <c r="T177" s="6" t="n"/>
     </row>
     <row r="178">
       <c r="A178" s="6" t="n"/>
@@ -4526,6 +4715,7 @@
       <c r="Q178" s="6" t="n"/>
       <c r="R178" s="6" t="n"/>
       <c r="S178" s="6" t="n"/>
+      <c r="T178" s="6" t="n"/>
     </row>
     <row r="179">
       <c r="A179" s="6" t="n"/>
@@ -4547,6 +4737,7 @@
       <c r="Q179" s="6" t="n"/>
       <c r="R179" s="6" t="n"/>
       <c r="S179" s="6" t="n"/>
+      <c r="T179" s="6" t="n"/>
     </row>
     <row r="180">
       <c r="A180" s="6" t="n"/>
@@ -4568,6 +4759,7 @@
       <c r="Q180" s="6" t="n"/>
       <c r="R180" s="6" t="n"/>
       <c r="S180" s="6" t="n"/>
+      <c r="T180" s="6" t="n"/>
     </row>
     <row r="181">
       <c r="A181" s="6" t="n"/>
@@ -4589,6 +4781,7 @@
       <c r="Q181" s="6" t="n"/>
       <c r="R181" s="6" t="n"/>
       <c r="S181" s="6" t="n"/>
+      <c r="T181" s="6" t="n"/>
     </row>
     <row r="182">
       <c r="A182" s="6" t="n"/>
@@ -4610,6 +4803,7 @@
       <c r="Q182" s="6" t="n"/>
       <c r="R182" s="6" t="n"/>
       <c r="S182" s="6" t="n"/>
+      <c r="T182" s="6" t="n"/>
     </row>
     <row r="183">
       <c r="A183" s="6" t="n"/>
@@ -4631,6 +4825,7 @@
       <c r="Q183" s="6" t="n"/>
       <c r="R183" s="6" t="n"/>
       <c r="S183" s="6" t="n"/>
+      <c r="T183" s="6" t="n"/>
     </row>
     <row r="184">
       <c r="A184" s="6" t="n"/>
@@ -4652,6 +4847,7 @@
       <c r="Q184" s="6" t="n"/>
       <c r="R184" s="6" t="n"/>
       <c r="S184" s="6" t="n"/>
+      <c r="T184" s="6" t="n"/>
     </row>
     <row r="185">
       <c r="A185" s="6" t="n"/>
@@ -4673,6 +4869,7 @@
       <c r="Q185" s="6" t="n"/>
       <c r="R185" s="6" t="n"/>
       <c r="S185" s="6" t="n"/>
+      <c r="T185" s="6" t="n"/>
     </row>
     <row r="186">
       <c r="A186" s="6" t="n"/>
@@ -4694,6 +4891,7 @@
       <c r="Q186" s="6" t="n"/>
       <c r="R186" s="6" t="n"/>
       <c r="S186" s="6" t="n"/>
+      <c r="T186" s="6" t="n"/>
     </row>
     <row r="187">
       <c r="A187" s="6" t="n"/>
@@ -4715,6 +4913,7 @@
       <c r="Q187" s="6" t="n"/>
       <c r="R187" s="6" t="n"/>
       <c r="S187" s="6" t="n"/>
+      <c r="T187" s="6" t="n"/>
     </row>
     <row r="188">
       <c r="A188" s="6" t="n"/>
@@ -4736,6 +4935,7 @@
       <c r="Q188" s="6" t="n"/>
       <c r="R188" s="6" t="n"/>
       <c r="S188" s="6" t="n"/>
+      <c r="T188" s="6" t="n"/>
     </row>
     <row r="189">
       <c r="A189" s="6" t="n"/>
@@ -4757,6 +4957,7 @@
       <c r="Q189" s="6" t="n"/>
       <c r="R189" s="6" t="n"/>
       <c r="S189" s="6" t="n"/>
+      <c r="T189" s="6" t="n"/>
     </row>
     <row r="190">
       <c r="A190" s="6" t="n"/>
@@ -4778,6 +4979,7 @@
       <c r="Q190" s="6" t="n"/>
       <c r="R190" s="6" t="n"/>
       <c r="S190" s="6" t="n"/>
+      <c r="T190" s="6" t="n"/>
     </row>
     <row r="191">
       <c r="A191" s="6" t="n"/>
@@ -4799,6 +5001,7 @@
       <c r="Q191" s="6" t="n"/>
       <c r="R191" s="6" t="n"/>
       <c r="S191" s="6" t="n"/>
+      <c r="T191" s="6" t="n"/>
     </row>
     <row r="192">
       <c r="A192" s="6" t="n"/>
@@ -4820,6 +5023,7 @@
       <c r="Q192" s="6" t="n"/>
       <c r="R192" s="6" t="n"/>
       <c r="S192" s="6" t="n"/>
+      <c r="T192" s="6" t="n"/>
     </row>
     <row r="193">
       <c r="A193" s="6" t="n"/>
@@ -4841,6 +5045,7 @@
       <c r="Q193" s="6" t="n"/>
       <c r="R193" s="6" t="n"/>
       <c r="S193" s="6" t="n"/>
+      <c r="T193" s="6" t="n"/>
     </row>
     <row r="194">
       <c r="A194" s="6" t="n"/>
@@ -4862,6 +5067,7 @@
       <c r="Q194" s="6" t="n"/>
       <c r="R194" s="6" t="n"/>
       <c r="S194" s="6" t="n"/>
+      <c r="T194" s="6" t="n"/>
     </row>
     <row r="195">
       <c r="A195" s="6" t="n"/>
@@ -4883,6 +5089,7 @@
       <c r="Q195" s="6" t="n"/>
       <c r="R195" s="6" t="n"/>
       <c r="S195" s="6" t="n"/>
+      <c r="T195" s="6" t="n"/>
     </row>
     <row r="196">
       <c r="A196" s="6" t="n"/>
@@ -4904,6 +5111,7 @@
       <c r="Q196" s="6" t="n"/>
       <c r="R196" s="6" t="n"/>
       <c r="S196" s="6" t="n"/>
+      <c r="T196" s="6" t="n"/>
     </row>
     <row r="197">
       <c r="A197" s="6" t="n"/>
@@ -4925,6 +5133,7 @@
       <c r="Q197" s="6" t="n"/>
       <c r="R197" s="6" t="n"/>
       <c r="S197" s="6" t="n"/>
+      <c r="T197" s="6" t="n"/>
     </row>
     <row r="198">
       <c r="A198" s="6" t="n"/>
@@ -4946,6 +5155,7 @@
       <c r="Q198" s="6" t="n"/>
       <c r="R198" s="6" t="n"/>
       <c r="S198" s="6" t="n"/>
+      <c r="T198" s="6" t="n"/>
     </row>
     <row r="199">
       <c r="A199" s="6" t="n"/>
@@ -4967,6 +5177,7 @@
       <c r="Q199" s="6" t="n"/>
       <c r="R199" s="6" t="n"/>
       <c r="S199" s="6" t="n"/>
+      <c r="T199" s="6" t="n"/>
     </row>
     <row r="200">
       <c r="A200" s="6" t="n"/>
@@ -4988,6 +5199,7 @@
       <c r="Q200" s="6" t="n"/>
       <c r="R200" s="6" t="n"/>
       <c r="S200" s="6" t="n"/>
+      <c r="T200" s="6" t="n"/>
     </row>
     <row r="201">
       <c r="A201" s="6" t="n"/>
@@ -5009,6 +5221,7 @@
       <c r="Q201" s="6" t="n"/>
       <c r="R201" s="6" t="n"/>
       <c r="S201" s="6" t="n"/>
+      <c r="T201" s="6" t="n"/>
     </row>
     <row r="202">
       <c r="A202" s="6" t="n"/>
@@ -5030,6 +5243,7 @@
       <c r="Q202" s="6" t="n"/>
       <c r="R202" s="6" t="n"/>
       <c r="S202" s="6" t="n"/>
+      <c r="T202" s="6" t="n"/>
     </row>
     <row r="203">
       <c r="A203" s="6" t="n"/>
@@ -5051,6 +5265,7 @@
       <c r="Q203" s="6" t="n"/>
       <c r="R203" s="6" t="n"/>
       <c r="S203" s="6" t="n"/>
+      <c r="T203" s="6" t="n"/>
     </row>
     <row r="204">
       <c r="A204" s="6" t="n"/>
@@ -5072,6 +5287,7 @@
       <c r="Q204" s="6" t="n"/>
       <c r="R204" s="6" t="n"/>
       <c r="S204" s="6" t="n"/>
+      <c r="T204" s="6" t="n"/>
     </row>
     <row r="205">
       <c r="A205" s="6" t="n"/>
@@ -5093,21 +5309,22 @@
       <c r="Q205" s="6" t="n"/>
       <c r="R205" s="6" t="n"/>
       <c r="S205" s="6" t="n"/>
+      <c r="T205" s="6" t="n"/>
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="1" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="0" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="0" formatRows="1" sort="0"/>
   <mergeCells count="2">
-    <mergeCell ref="A2:S2"/>
-    <mergeCell ref="A1:S1"/>
+    <mergeCell ref="A1:T1"/>
+    <mergeCell ref="A2:T2"/>
   </mergeCells>
   <dataValidations count="3">
-    <dataValidation sqref="D5:D205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Choose a value from the dropdown for Course Type." promptTitle="Course Type" prompt="Select a Course Type from the list." type="list">
+    <dataValidation sqref="E5:E205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Choose a value from the dropdown for Course Type." promptTitle="Course Type" prompt="Select a Course Type from the list." type="list">
       <formula1>=Lists!$A$2:$A$7</formula1>
     </dataValidation>
-    <dataValidation sqref="G5:G205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Choose a value from the dropdown for Time Zone." promptTitle="Time Zone" prompt="Select a Time Zone from the list." type="list">
+    <dataValidation sqref="H5:H205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Choose a value from the dropdown for Time Zone." promptTitle="Time Zone" prompt="Select a Time Zone from the list." type="list">
       <formula1>=Lists!$B$2:$B$6</formula1>
     </dataValidation>
-    <dataValidation sqref="O5:O205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Choose a value from the dropdown for State." promptTitle="State" prompt="Select a State from the list." type="list">
+    <dataValidation sqref="P5:P205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Choose a value from the dropdown for State." promptTitle="State" prompt="Select a State from the list." type="list">
       <formula1>=Lists!$C$2:$C$53</formula1>
     </dataValidation>
   </dataValidations>
@@ -5122,7 +5339,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C34"/>
+  <dimension ref="A1:C36"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5168,65 +5385,55 @@
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>•  Provider and Country are set automatically on upload, so they are not in this sheet.</t>
-        </is>
-      </c>
-    </row>
-    <row r="9">
-      <c r="A9" s="8" t="inlineStr">
+          <t>•  Provider must exactly match an existing provider name; leave it blank to use your own provider.</t>
+        </is>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="7" t="inlineStr">
+        <is>
+          <t>•  Country is always US and is set automatically, so it is not in this sheet.</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" s="8" t="inlineStr">
         <is>
           <t>Column</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>Required</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>Description &amp; accepted values</t>
-        </is>
-      </c>
-    </row>
-    <row r="10" ht="30" customHeight="1">
-      <c r="A10" s="9" t="inlineStr">
-        <is>
-          <t>Title</t>
-        </is>
-      </c>
-      <c r="B10" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
-        </is>
-      </c>
-      <c r="C10" s="11" t="inlineStr">
-        <is>
-          <t>The public name of the course. Required.</t>
         </is>
       </c>
     </row>
     <row r="11" ht="30" customHeight="1">
       <c r="A11" s="9" t="inlineStr">
         <is>
-          <t>Subtitle</t>
-        </is>
-      </c>
-      <c r="B11" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Title</t>
+        </is>
+      </c>
+      <c r="B11" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Optional tagline shown under the title.</t>
+          <t>The public name of the course. Required.</t>
         </is>
       </c>
     </row>
     <row r="12" ht="30" customHeight="1">
       <c r="A12" s="9" t="inlineStr">
         <is>
-          <t>Description</t>
+          <t>Subtitle</t>
         </is>
       </c>
       <c r="B12" s="12" t="inlineStr">
@@ -5236,48 +5443,48 @@
       </c>
       <c r="C12" s="11" t="inlineStr">
         <is>
-          <t>Short summary shown in course previews.</t>
+          <t>Optional tagline shown under the title.</t>
         </is>
       </c>
     </row>
     <row r="13" ht="30" customHeight="1">
       <c r="A13" s="9" t="inlineStr">
         <is>
-          <t>Course Type</t>
-        </is>
-      </c>
-      <c r="B13" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Description</t>
+        </is>
+      </c>
+      <c r="B13" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Choose one from the dropdown. Required.</t>
+          <t>Short summary shown in course previews.</t>
         </is>
       </c>
     </row>
     <row r="14" ht="30" customHeight="1">
       <c r="A14" s="9" t="inlineStr">
         <is>
-          <t>Start Date</t>
-        </is>
-      </c>
-      <c r="B14" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Provider</t>
+        </is>
+      </c>
+      <c r="B14" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>Format MM/DD/YYYY. Required.</t>
+          <t>The provider/organization offering the course. Must exactly match an existing provider name. Leave blank to use the uploader's own provider.</t>
         </is>
       </c>
     </row>
     <row r="15" ht="30" customHeight="1">
       <c r="A15" s="9" t="inlineStr">
         <is>
-          <t>Start Time</t>
+          <t>Course Type</t>
         </is>
       </c>
       <c r="B15" s="10" t="inlineStr">
@@ -5287,14 +5494,14 @@
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Format H:MM AM/PM, e.g. 9:00 AM. Required.</t>
+          <t>Choose one from the dropdown. Required.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="30" customHeight="1">
       <c r="A16" s="9" t="inlineStr">
         <is>
-          <t>Time Zone</t>
+          <t>Start Date</t>
         </is>
       </c>
       <c r="B16" s="10" t="inlineStr">
@@ -5304,48 +5511,48 @@
       </c>
       <c r="C16" s="11" t="inlineStr">
         <is>
-          <t>Choose one from the dropdown. Applies to all times in the row. Required.</t>
+          <t>Format MM/DD/YYYY. Required.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="30" customHeight="1">
       <c r="A17" s="9" t="inlineStr">
         <is>
-          <t>End Date</t>
-        </is>
-      </c>
-      <c r="B17" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Start Time</t>
+        </is>
+      </c>
+      <c r="B17" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Optional. For multi-day courses. MM/DD/YYYY.</t>
+          <t>Format H:MM AM/PM, e.g. 9:00 AM. Required.</t>
         </is>
       </c>
     </row>
     <row r="18" ht="30" customHeight="1">
       <c r="A18" s="9" t="inlineStr">
         <is>
-          <t>End Time</t>
-        </is>
-      </c>
-      <c r="B18" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Time Zone</t>
+        </is>
+      </c>
+      <c r="B18" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C18" s="11" t="inlineStr">
         <is>
-          <t>Optional. H:MM AM/PM.</t>
+          <t>Choose one from the dropdown. Applies to all times in the row. Required.</t>
         </is>
       </c>
     </row>
     <row r="19" ht="30" customHeight="1">
       <c r="A19" s="9" t="inlineStr">
         <is>
-          <t>Registration Deadline Date</t>
+          <t>End Date</t>
         </is>
       </c>
       <c r="B19" s="12" t="inlineStr">
@@ -5355,14 +5562,14 @@
       </c>
       <c r="C19" s="11" t="inlineStr">
         <is>
-          <t>Optional. Must be before Start Date. MM/DD/YYYY.</t>
+          <t>Optional. For multi-day courses. MM/DD/YYYY.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="30" customHeight="1">
       <c r="A20" s="9" t="inlineStr">
         <is>
-          <t>Registration Deadline Time</t>
+          <t>End Time</t>
         </is>
       </c>
       <c r="B20" s="12" t="inlineStr">
@@ -5379,24 +5586,24 @@
     <row r="21" ht="30" customHeight="1">
       <c r="A21" s="9" t="inlineStr">
         <is>
-          <t>Place Name</t>
-        </is>
-      </c>
-      <c r="B21" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Registration Deadline Date</t>
+        </is>
+      </c>
+      <c r="B21" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="C21" s="11" t="inlineStr">
         <is>
-          <t>Venue or meeting place name. Required.</t>
+          <t>Optional. Must be before Start Date. MM/DD/YYYY.</t>
         </is>
       </c>
     </row>
     <row r="22" ht="30" customHeight="1">
       <c r="A22" s="9" t="inlineStr">
         <is>
-          <t>Street Address</t>
+          <t>Registration Deadline Time</t>
         </is>
       </c>
       <c r="B22" s="12" t="inlineStr">
@@ -5406,48 +5613,48 @@
       </c>
       <c r="C22" s="11" t="inlineStr">
         <is>
-          <t>Optional street address.</t>
+          <t>Optional. H:MM AM/PM.</t>
         </is>
       </c>
     </row>
     <row r="23" ht="30" customHeight="1">
       <c r="A23" s="9" t="inlineStr">
         <is>
-          <t>City</t>
-        </is>
-      </c>
-      <c r="B23" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>Place Name</t>
+        </is>
+      </c>
+      <c r="B23" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C23" s="11" t="inlineStr">
         <is>
-          <t>Optional.</t>
+          <t>Venue or meeting place name. Required.</t>
         </is>
       </c>
     </row>
     <row r="24" ht="30" customHeight="1">
       <c r="A24" s="9" t="inlineStr">
         <is>
-          <t>State</t>
-        </is>
-      </c>
-      <c r="B24" s="10" t="inlineStr">
-        <is>
-          <t>Yes</t>
+          <t>Street Address</t>
+        </is>
+      </c>
+      <c r="B24" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
         </is>
       </c>
       <c r="C24" s="11" t="inlineStr">
         <is>
-          <t>Two-letter code from dropdown. Required.</t>
+          <t>Optional street address.</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="9" t="inlineStr">
         <is>
-          <t>ZIP Code</t>
+          <t>City</t>
         </is>
       </c>
       <c r="B25" s="12" t="inlineStr">
@@ -5457,31 +5664,31 @@
       </c>
       <c r="C25" s="11" t="inlineStr">
         <is>
-          <t>Optional. 5 digits (or 5+4).</t>
+          <t>Optional.</t>
         </is>
       </c>
     </row>
     <row r="26" ht="30" customHeight="1">
       <c r="A26" s="9" t="inlineStr">
         <is>
-          <t>Course URL</t>
-        </is>
-      </c>
-      <c r="B26" s="12" t="inlineStr">
-        <is>
-          <t>No</t>
+          <t>State</t>
+        </is>
+      </c>
+      <c r="B26" s="10" t="inlineStr">
+        <is>
+          <t>Yes</t>
         </is>
       </c>
       <c r="C26" s="11" t="inlineStr">
         <is>
-          <t>Optional. Full registration/landing link starting with https://</t>
+          <t>Two-letter code from dropdown. Required.</t>
         </is>
       </c>
     </row>
     <row r="27" ht="30" customHeight="1">
       <c r="A27" s="9" t="inlineStr">
         <is>
-          <t>Mode of Travel</t>
+          <t>ZIP Code</t>
         </is>
       </c>
       <c r="B27" s="12" t="inlineStr">
@@ -5491,82 +5698,116 @@
       </c>
       <c r="C27" s="11" t="inlineStr">
         <is>
-          <t>Optional. One or more of: Ski, Splitboard, Motorized, Snowshoe. Separate multiple with commas.</t>
+          <t>Optional. 5 digits (or 5+4).</t>
         </is>
       </c>
     </row>
     <row r="28" ht="30" customHeight="1">
       <c r="A28" s="9" t="inlineStr">
         <is>
+          <t>Course URL</t>
+        </is>
+      </c>
+      <c r="B28" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C28" s="11" t="inlineStr">
+        <is>
+          <t>Optional. Full registration/landing link starting with https://</t>
+        </is>
+      </c>
+    </row>
+    <row r="29" ht="30" customHeight="1">
+      <c r="A29" s="9" t="inlineStr">
+        <is>
+          <t>Mode of Travel</t>
+        </is>
+      </c>
+      <c r="B29" s="12" t="inlineStr">
+        <is>
+          <t>No</t>
+        </is>
+      </c>
+      <c r="C29" s="11" t="inlineStr">
+        <is>
+          <t>Optional. One or more of: Ski, Splitboard, Motorized, Snowshoe. Separate multiple with commas.</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="30" customHeight="1">
+      <c r="A30" s="9" t="inlineStr">
+        <is>
           <t>Interest Groups</t>
         </is>
       </c>
-      <c r="B28" s="12" t="inlineStr">
+      <c r="B30" s="12" t="inlineStr">
         <is>
           <t>No</t>
         </is>
       </c>
-      <c r="C28" s="11" t="inlineStr">
+      <c r="C30" s="11" t="inlineStr">
         <is>
           <t>Optional. One or more of: For LGBTQ+, For Women, For Youth. Separate multiple with commas.</t>
-        </is>
-      </c>
-    </row>
-    <row r="30" ht="30" customHeight="1">
-      <c r="A30" s="13" t="inlineStr">
-        <is>
-          <t>Course Type options</t>
-        </is>
-      </c>
-      <c r="B30" s="14" t="inlineStr">
-        <is>
-          <t>Rec 1, Rec 2, Pro 1, Pro 2, Rescue, Awareness</t>
-        </is>
-      </c>
-    </row>
-    <row r="31" ht="30" customHeight="1">
-      <c r="A31" s="13" t="inlineStr">
-        <is>
-          <t>Time Zone options</t>
-        </is>
-      </c>
-      <c r="B31" s="14" t="inlineStr">
-        <is>
-          <t>Eastern Time (ET), Mountain Time (MT), Pacific Time (PT), Alaska Time (AKT), Island Time (HT)</t>
         </is>
       </c>
     </row>
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Mode of Travel options</t>
+          <t>Course Type options</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Ski, Splitboard, Motorized, Snowshoe  (comma-separate multiple)</t>
+          <t>Rec 1, Rec 2, Pro 1, Pro 2, Rescue, Awareness</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>Interest Groups options</t>
+          <t>Time Zone options</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>For LGBTQ+, For Women, For Youth  (comma-separate multiple)</t>
+          <t>Eastern Time (ET), Mountain Time (MT), Pacific Time (PT), Alaska Time (AKT), Island Time (HT)</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
+          <t>Mode of Travel options</t>
+        </is>
+      </c>
+      <c r="B34" s="14" t="inlineStr">
+        <is>
+          <t>Ski, Splitboard, Motorized, Snowshoe  (comma-separate multiple)</t>
+        </is>
+      </c>
+    </row>
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="13" t="inlineStr">
+        <is>
+          <t>Interest Groups options</t>
+        </is>
+      </c>
+      <c r="B35" s="14" t="inlineStr">
+        <is>
+          <t>For LGBTQ+, For Women, For Youth  (comma-separate multiple)</t>
+        </is>
+      </c>
+    </row>
+    <row r="36" ht="30" customHeight="1">
+      <c r="A36" s="13" t="inlineStr">
+        <is>
           <t>State options</t>
         </is>
       </c>
-      <c r="B34" s="14" t="inlineStr">
+      <c r="B36" s="14" t="inlineStr">
         <is>
           <t>AL, AK, AZ, AR, CA, CO, CT, DE, FL, GA, HI, ID, IL, IN, IA, KS, KY, LA, ME, MD, MA, MI, MN, MS, MO, MT, NE, NV, NH, NJ, NM, NY, NC, ND, OH, OK, OR, PA, RI, SC, SD, TN, TX, UT, VT, VA, WA, WV, WI, WY, DC, International</t>
         </is>
@@ -5574,18 +5815,19 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="11">
-    <mergeCell ref="B30:C30"/>
+  <mergeCells count="12">
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
+    <mergeCell ref="A8:C8"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="A6:C6"/>
+    <mergeCell ref="B36:C36"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A7:C7"/>
-    <mergeCell ref="B31:C31"/>
     <mergeCell ref="B32:C32"/>
     <mergeCell ref="A4:C4"/>
+    <mergeCell ref="B35:C35"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Make Provider a dropdown in course upload template
Convert the Provider column from free text to a dropdown populated from
the available providers (seeded provider set). Update the example row,
Instructions tab, and accepted-values appendix accordingly.

Co-Authored-By: Claude Opus 4.8 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Y8EAvR5NE5imEw4oAyMGQu
</commit_message>
<xml_diff>
--- a/Course-Records-Upload-Template.xlsx
+++ b/Course-Records-Upload-Template.xlsx
@@ -265,7 +265,7 @@
     </comment>
     <comment ref="D3" authorId="0" shapeId="0">
       <text>
-        <t>The provider/organization offering the course. Must exactly match an existing provider name. Leave blank to use the uploader's own provider.</t>
+        <t>The provider/organization offering the course. Choose one from the dropdown. Leave blank to use the uploader's own provider.</t>
       </text>
     </comment>
     <comment ref="E3" authorId="0" shapeId="0">
@@ -652,7 +652,7 @@
     <col width="32" customWidth="1" min="1" max="1"/>
     <col width="26" customWidth="1" min="2" max="2"/>
     <col width="40" customWidth="1" min="3" max="3"/>
-    <col width="24" customWidth="1" min="4" max="4"/>
+    <col width="26" customWidth="1" min="4" max="4"/>
     <col width="16" customWidth="1" min="5" max="5"/>
     <col width="14" customWidth="1" min="6" max="6"/>
     <col width="12" customWidth="1" min="7" max="7"/>
@@ -805,7 +805,7 @@
       </c>
       <c r="D4" s="5" t="inlineStr">
         <is>
-          <t>Northwest Avalanche Institute</t>
+          <t>Mountain Education Center</t>
         </is>
       </c>
       <c r="E4" s="5" t="inlineStr">
@@ -5317,7 +5317,7 @@
     <mergeCell ref="A1:T1"/>
     <mergeCell ref="A2:T2"/>
   </mergeCells>
-  <dataValidations count="3">
+  <dataValidations count="4">
     <dataValidation sqref="E5:E205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Choose a value from the dropdown for Course Type." promptTitle="Course Type" prompt="Select a Course Type from the list." type="list">
       <formula1>=Lists!$A$2:$A$7</formula1>
     </dataValidation>
@@ -5326,6 +5326,9 @@
     </dataValidation>
     <dataValidation sqref="P5:P205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Choose a value from the dropdown for State." promptTitle="State" prompt="Select a State from the list." type="list">
       <formula1>=Lists!$C$2:$C$53</formula1>
+    </dataValidation>
+    <dataValidation sqref="D5:D205" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="1" errorTitle="Invalid entry" error="Choose a value from the dropdown for Provider." promptTitle="Provider" prompt="Select a Provider from the list." type="list">
+      <formula1>=Lists!$F$2:$F$5</formula1>
     </dataValidation>
   </dataValidations>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -5339,7 +5342,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C36"/>
+  <dimension ref="A1:C37"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="30" customWidth="1" min="1" max="1"/>
@@ -5378,14 +5381,14 @@
     <row r="6">
       <c r="A6" s="7" t="inlineStr">
         <is>
-          <t>•  Course Type, Time Zone, and State use dropdowns — click the cell and pick a value.</t>
+          <t>•  Provider, Course Type, Time Zone, and State use dropdowns — click the cell and pick a value.</t>
         </is>
       </c>
     </row>
     <row r="7">
       <c r="A7" s="7" t="inlineStr">
         <is>
-          <t>•  Provider must exactly match an existing provider name; leave it blank to use your own provider.</t>
+          <t>•  Leave Provider blank to use your own provider.</t>
         </is>
       </c>
     </row>
@@ -5477,7 +5480,7 @@
       </c>
       <c r="C14" s="11" t="inlineStr">
         <is>
-          <t>The provider/organization offering the course. Must exactly match an existing provider name. Leave blank to use the uploader's own provider.</t>
+          <t>The provider/organization offering the course. Choose one from the dropdown. Leave blank to use the uploader's own provider.</t>
         </is>
       </c>
     </row>
@@ -5756,58 +5759,70 @@
     <row r="32" ht="30" customHeight="1">
       <c r="A32" s="13" t="inlineStr">
         <is>
-          <t>Course Type options</t>
+          <t>Provider options</t>
         </is>
       </c>
       <c r="B32" s="14" t="inlineStr">
         <is>
-          <t>Rec 1, Rec 2, Pro 1, Pro 2, Rescue, Awareness</t>
+          <t>Alpine Skills International, Backcountry Alliance, Mountain Education Center, Pro Avalanche Training</t>
         </is>
       </c>
     </row>
     <row r="33" ht="30" customHeight="1">
       <c r="A33" s="13" t="inlineStr">
         <is>
-          <t>Time Zone options</t>
+          <t>Course Type options</t>
         </is>
       </c>
       <c r="B33" s="14" t="inlineStr">
         <is>
-          <t>Eastern Time (ET), Mountain Time (MT), Pacific Time (PT), Alaska Time (AKT), Island Time (HT)</t>
+          <t>Rec 1, Rec 2, Pro 1, Pro 2, Rescue, Awareness</t>
         </is>
       </c>
     </row>
     <row r="34" ht="30" customHeight="1">
       <c r="A34" s="13" t="inlineStr">
         <is>
-          <t>Mode of Travel options</t>
+          <t>Time Zone options</t>
         </is>
       </c>
       <c r="B34" s="14" t="inlineStr">
         <is>
-          <t>Ski, Splitboard, Motorized, Snowshoe  (comma-separate multiple)</t>
+          <t>Eastern Time (ET), Mountain Time (MT), Pacific Time (PT), Alaska Time (AKT), Island Time (HT)</t>
         </is>
       </c>
     </row>
     <row r="35" ht="30" customHeight="1">
       <c r="A35" s="13" t="inlineStr">
         <is>
-          <t>Interest Groups options</t>
+          <t>Mode of Travel options</t>
         </is>
       </c>
       <c r="B35" s="14" t="inlineStr">
         <is>
-          <t>For LGBTQ+, For Women, For Youth  (comma-separate multiple)</t>
+          <t>Ski, Splitboard, Motorized, Snowshoe  (comma-separate multiple)</t>
         </is>
       </c>
     </row>
     <row r="36" ht="30" customHeight="1">
       <c r="A36" s="13" t="inlineStr">
         <is>
+          <t>Interest Groups options</t>
+        </is>
+      </c>
+      <c r="B36" s="14" t="inlineStr">
+        <is>
+          <t>For LGBTQ+, For Women, For Youth  (comma-separate multiple)</t>
+        </is>
+      </c>
+    </row>
+    <row r="37" ht="30" customHeight="1">
+      <c r="A37" s="13" t="inlineStr">
+        <is>
           <t>State options</t>
         </is>
       </c>
-      <c r="B36" s="14" t="inlineStr">
+      <c r="B37" s="14" t="inlineStr">
         <is>
           <t>AL, AK, AZ, AR, CA, CO, CT, DE, FL, GA, HI, ID, IL, IN, IA, KS, KY, LA, ME, MD, MA, MI, MN, MS, MO, MT, NE, NV, NH, NJ, NM, NY, NC, ND, OH, OK, OR, PA, RI, SC, SD, TN, TX, UT, VT, VA, WA, WV, WI, WY, DC, International</t>
         </is>
@@ -5815,13 +5830,14 @@
     </row>
   </sheetData>
   <sheetProtection selectLockedCells="1" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
-  <mergeCells count="12">
+  <mergeCells count="13">
     <mergeCell ref="B33:C33"/>
     <mergeCell ref="A1:C1"/>
     <mergeCell ref="A5:C5"/>
     <mergeCell ref="A8:C8"/>
     <mergeCell ref="B34:C34"/>
     <mergeCell ref="A6:C6"/>
+    <mergeCell ref="B37:C37"/>
     <mergeCell ref="B36:C36"/>
     <mergeCell ref="A3:C3"/>
     <mergeCell ref="A7:C7"/>
@@ -5839,7 +5855,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E53"/>
+  <dimension ref="A1:F53"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -5868,6 +5884,11 @@
           <t>InterestGroup</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>Provider</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -5895,6 +5916,11 @@
           <t>For LGBTQ+</t>
         </is>
       </c>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>Alpine Skills International</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -5922,6 +5948,11 @@
           <t>For Women</t>
         </is>
       </c>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>Backcountry Alliance</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -5949,6 +5980,11 @@
           <t>For Youth</t>
         </is>
       </c>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>Mountain Education Center</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -5969,6 +6005,11 @@
       <c r="D5" t="inlineStr">
         <is>
           <t>Snowshoe</t>
+        </is>
+      </c>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Pro Avalanche Training</t>
         </is>
       </c>
     </row>

</xml_diff>